<commit_message>
Add comprehensive RUM browser regression suites
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/RUM_Performance_Details_Regression.xlsx
+++ b/docs/RUM_Performance_Details_Regression.xlsx
@@ -13,9 +13,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="204">
-  <si>
-    <t>Profile: US / GDC Test Site 2 | Type: Regression (read-only) | Total TCs: 36 | RUM Performance Detail</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="415" uniqueCount="222">
+  <si>
+    <t>Profile: US / GDC Test Site 2 | Type: Regression (read-only) | Total TCs: 40 | RUM Performance Detail</t>
   </si>
   <si>
     <t>Confluence: https://bluetriangletech.atlassian.net/wiki/spaces/HCT/pages/3186720883/RUM+Performance+Detail+Page</t>
@@ -45,13 +45,13 @@
     <t>(all)</t>
   </si>
   <si>
-    <t>REG-RUM-PD-001, REG-RUM-PD-002, REG-RUM-PD-003, REG-RUM-PD-004, REG-RUM-PD-005, REG-RUM-PD-006, REG-RUM-PD-007, REG-RUM-PD-008, REG-RUM-PD-009, REG-RUM-PD-010, REG-RUM-PD-011, REG-RUM-PD-012, REG-RUM-PD-013, REG-RUM-PD-014, REG-RUM-PD-015, REG-RUM-PD-016, REG-RUM-PD-017, REG-RUM-PD-018, REG-RUM-PD-019, REG-RUM-PD-020, REG-RUM-PD-021, REG-RUM-PD-022, REG-RUM-PD-023, REG-RUM-PD-024, REG-RUM-PD-025, REG-RUM-PD-026, REG-RUM-PD-027, REG-RUM-PD-028, REG-RUM-PD-029, REG-RUM-PD-030, REG-RUM-PD-031, REG-RUM-PD-032, REG-RUM-PD-033, REG-RUM-PD-034, REG-RUM-PD-035, REG-RUM-PD-036</t>
+    <t>REG-RUM-PD-001, REG-RUM-PD-002, REG-RUM-PD-003, REG-RUM-PD-004, REG-RUM-PD-005, REG-RUM-PD-006, REG-RUM-PD-007, REG-RUM-PD-008, REG-RUM-PD-009, REG-RUM-PD-010, REG-RUM-PD-011, REG-RUM-PD-012, REG-RUM-PD-013, REG-RUM-PD-014, REG-RUM-PD-015, REG-RUM-PD-016, REG-RUM-PD-017, REG-RUM-PD-018, REG-RUM-PD-019, REG-RUM-PD-020, REG-RUM-PD-021, REG-RUM-PD-022, REG-RUM-PD-023, REG-RUM-PD-024, REG-RUM-PD-025, REG-RUM-PD-026, REG-RUM-PD-027, REG-RUM-PD-028, REG-RUM-PD-029, REG-RUM-PD-030, REG-RUM-PD-031, REG-RUM-PD-032, REG-RUM-PD-033, REG-RUM-PD-034, REG-RUM-PD-035, REG-RUM-PD-036, REG-RUM-PD-037, REG-RUM-PD-038, REG-RUM-PD-039, REG-RUM-PD-040</t>
   </si>
   <si>
     <t>TOTAL</t>
   </si>
   <si>
-    <t>REG-RUM-PD-001 .. REG-RUM-PD-036</t>
+    <t>REG-RUM-PD-001 .. REG-RUM-PD-040</t>
   </si>
   <si>
     <t>Breakdown by Module + Submodule</t>
@@ -61,6 +61,12 @@
   </si>
   <si>
     <t>REG-RUM-PD-007, REG-RUM-PD-008, REG-RUM-PD-009, REG-RUM-PD-013, REG-RUM-PD-014, REG-RUM-PD-034</t>
+  </si>
+  <si>
+    <t>Time Period / Bucket Size</t>
+  </si>
+  <si>
+    <t>REG-RUM-PD-037, REG-RUM-PD-038, REG-RUM-PD-039, REG-RUM-PD-040</t>
   </si>
   <si>
     <t>Filters</t>
@@ -752,6 +758,82 @@
 Charts refresh; missing bars for sparse data are noted</t>
   </si>
   <si>
+    <t>REG-RUM-PD-037</t>
+  </si>
+  <si>
+    <t>REG-RUM-PD-037 — Time Period Last 6 hours with Auto bucket on Perf Details + Page Timings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open right-nav Filters on RUM Performance Detail
+2. Set Time Period to Last 6 hours
+3. Keep Bucket Size = Auto (do not force a fixed bucket)
+4. Apply Filters (do NOT Save Filter)
+5. Confirm Performance Details and Page Timings Over Time are visible
+6. Hover Page Timings left→right (optional tooltips)
+7. Validate Highcharts x-axis spacing (~1 minute when Auto resolves for this window)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bucket Size remains Auto for the selected Time Period
+Performance Details + Page Timings refresh with chart data
+Timeline end is near local now; Auto typically resolves to ~1 minute buckets for Last 6 hours
+No Save Filter write is performed</t>
+  </si>
+  <si>
+    <t>REG-RUM-PD-038</t>
+  </si>
+  <si>
+    <t>REG-RUM-PD-038 — Time Period Last 24 hours with Auto bucket on Perf Details + Page Timings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Filters
+2. Set Time Period to Last 24 hours
+3. Keep Bucket Size = Auto
+4. Apply Filters
+5. Confirm Perf Details + Page Timings; validate timeline (~5 minute Auto buckets typical)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bucket Size stays Auto
+Charts refresh for Last 24 hours
+Auto typically resolves to ~5 minute buckets; end near now</t>
+  </si>
+  <si>
+    <t>REG-RUM-PD-039</t>
+  </si>
+  <si>
+    <t>REG-RUM-PD-039 — Time Period Last 7 days with Auto bucket on Perf Details + Page Timings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Filters
+2. Set Time Period to Last 7 days
+3. Keep Bucket Size = Auto
+4. Apply Filters
+5. Confirm Perf Details + Page Timings; validate timeline (~1 hour Auto buckets typical)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bucket Size stays Auto
+Charts refresh for Last 7 days
+Auto typically resolves to ~1 hour buckets; end near now</t>
+  </si>
+  <si>
+    <t>REG-RUM-PD-040</t>
+  </si>
+  <si>
+    <t>REG-RUM-PD-040 — Time Period Last 30 days with Auto bucket on Perf Details + Page Timings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open Filters
+2. Set Time Period to Last 30 days
+3. Keep Bucket Size = Auto
+4. Apply Filters
+5. Confirm Perf Details + Page Timings; validate timeline (~1 day Auto buckets typical)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bucket Size stays Auto
+Charts refresh for Last 30 days
+Auto typically resolves to ~1 day buckets; end near now
+Note: Bucket Size control exists on RUM Performance Detail Filters (not on Revenue Opportunity)</t>
+  </si>
+  <si>
     <t>Blue Triangle Portal — RUM Performance Detail (Browser) Regression Test Cases</t>
   </si>
   <si>
@@ -770,13 +852,13 @@
     <t>Excluded writes: Save Filter, Create Alert/Report, Create Custom Marker, Edit Profile, settings saves.</t>
   </si>
   <si>
-    <t>Total cases: 36 (REG-RUM-PD-001..REG-RUM-PD-036)</t>
+    <t>Total cases: 40 (REG-RUM-PD-001..REG-RUM-PD-040)</t>
   </si>
   <si>
     <t>Confluence reference: https://bluetriangletech.atlassian.net/wiki/spaces/HCT/pages/3186720883/RUM+Performance+Detail+Page</t>
   </si>
   <si>
-    <t>Automation mapping: tests/regression_tests/US2/rum.performance-detail.browser.regression.spec.ts</t>
+    <t>Automation mapping: tests/regression_tests/US2/monitoring/real-user-browser/performance-detail/rum.performance-detail.browser.regression.spec.ts</t>
   </si>
   <si>
     <t>Assumptions: metric/filter combos are sampled (not exhaustive); circle/triangle mix depends on live session data.</t>
@@ -1197,7 +1279,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="36" customWidth="1"/>
@@ -1258,7 +1340,7 @@
         <v>9</v>
       </c>
       <c r="D5" s="5">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>10</v>
@@ -1272,7 +1354,7 @@
         <v>7</v>
       </c>
       <c r="D6" s="6">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>12</v>
@@ -1314,7 +1396,7 @@
         <v>16</v>
       </c>
       <c r="D10" s="5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>17</v>
@@ -1370,7 +1452,7 @@
         <v>24</v>
       </c>
       <c r="D14" s="5">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E14" s="5" t="s">
         <v>25</v>
@@ -1440,7 +1522,7 @@
         <v>34</v>
       </c>
       <c r="D19" s="5">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E19" s="5" t="s">
         <v>35</v>
@@ -1542,6 +1624,20 @@
       </c>
       <c r="E26" s="5" t="s">
         <v>49</v>
+      </c>
+    </row>
+    <row r="27" spans="2:5" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="5">
+        <v>1</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -1556,7 +1652,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H37"/>
+  <dimension ref="A1:H41"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1570,10 +1666,10 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:8" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>2</v>
@@ -1582,180 +1678,180 @@
         <v>3</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H1" s="3" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="2" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="3" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C3" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F3" s="5" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="G3" s="5" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H3" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="4" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C4" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H4" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C5" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F5" s="5" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G5" s="5" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H5" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C6" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F6" s="5" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G6" s="5" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H6" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="7" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C7" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F7" s="5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="G7" s="5" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H7" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="8" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C8" s="5" t="s">
         <v>8</v>
@@ -1764,24 +1860,24 @@
         <v>14</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F8" s="5" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G8" s="5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H8" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="9" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C9" s="5" t="s">
         <v>8</v>
@@ -1790,24 +1886,24 @@
         <v>14</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H9" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="10" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C10" s="5" t="s">
         <v>8</v>
@@ -1816,102 +1912,102 @@
         <v>14</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="G10" s="5" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H10" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="11" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="G11" s="5" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H11" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="12" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G12" s="5" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="H12" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C13" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G13" s="5" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H13" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="14" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>8</v>
@@ -1920,24 +2016,24 @@
         <v>14</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G14" s="5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H14" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="15" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C15" s="5" t="s">
         <v>8</v>
@@ -1946,518 +2042,518 @@
         <v>14</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="G15" s="5" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H15" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="G16" s="5" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H16" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="G17" s="5" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H17" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="B18" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="G18" s="5" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H18" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B19" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E19" s="5" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="G19" s="5" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H19" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="20" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B20" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E20" s="5" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="G20" s="5" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H20" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="21" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="B21" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E21" s="5" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G21" s="5" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="H21" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="22" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="B22" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C22" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F22" s="5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="G22" s="5" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H22" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="23" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="B23" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E23" s="5" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F23" s="5" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G23" s="5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H23" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="B24" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E24" s="5" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F24" s="5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G24" s="5" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H24" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="25" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="B25" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="E25" s="5" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F25" s="5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="G25" s="5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H25" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="26" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="B26" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E26" s="5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="F26" s="5" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="G26" s="5" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H26" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="B27" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="F27" s="5" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="G27" s="5" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H27" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="28" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="G28" s="5" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H28" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="29" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B29" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="F29" s="5" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="G29" s="5" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H29" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="30" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="F30" s="5" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="G30" s="5" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H30" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="31" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B31" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F31" s="5" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="G31" s="5" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H31" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="32" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B32" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E32" s="5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="F32" s="5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="G32" s="5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H32" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="33" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="B33" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="E33" s="5" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="F33" s="5" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="G33" s="5" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="H33" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="34" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="B34" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E34" s="5" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="F34" s="5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="G34" s="5" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H34" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="B35" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>8</v>
@@ -2466,76 +2562,180 @@
         <v>14</v>
       </c>
       <c r="E35" s="5" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="F35" s="5" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="G35" s="5" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H35" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="36" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B36" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E36" s="5" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="F36" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="G36" s="5" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H36" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="37" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B37" s="5" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>8</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="E37" s="5" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="F37" s="5" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="G37" s="5" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="H37" s="5" t="s">
-        <v>60</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="38" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="5" t="s">
+        <v>196</v>
+      </c>
+      <c r="B38" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E38" s="5" t="s">
+        <v>197</v>
+      </c>
+      <c r="F38" s="5" t="s">
+        <v>198</v>
+      </c>
+      <c r="G38" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="H38" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="39" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>200</v>
+      </c>
+      <c r="B39" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C39" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D39" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E39" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="F39" s="5" t="s">
+        <v>202</v>
+      </c>
+      <c r="G39" s="5" t="s">
+        <v>203</v>
+      </c>
+      <c r="H39" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="40" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B40" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D40" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E40" s="5" t="s">
+        <v>205</v>
+      </c>
+      <c r="F40" s="5" t="s">
+        <v>206</v>
+      </c>
+      <c r="G40" s="5" t="s">
+        <v>207</v>
+      </c>
+      <c r="H40" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="41" ht="110" customHeight="1" spans="1:8" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="5" t="s">
+        <v>208</v>
+      </c>
+      <c r="B41" s="5" t="s">
+        <v>58</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D41" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E41" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="F41" s="5" t="s">
+        <v>210</v>
+      </c>
+      <c r="G41" s="5" t="s">
+        <v>211</v>
+      </c>
+      <c r="H41" s="5" t="s">
+        <v>62</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" sqref="H10:H37">
+    <dataValidation type="list" allowBlank="1" sqref="H10:H41">
       <formula1>"Not Executed,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="H2:H37">
+    <dataValidation type="list" allowBlank="1" sqref="H2:H41">
       <formula1>"Not Executed,Pass,Fail,Blocked,Skipped"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2554,52 +2754,52 @@
   <sheetData>
     <row r="1" spans="1:1" s="7" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>194</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>195</v>
+        <v>213</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>196</v>
+        <v>214</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>197</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>198</v>
+        <v>216</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>199</v>
+        <v>217</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>200</v>
+        <v>218</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>201</v>
+        <v>219</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>202</v>
+        <v>220</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>203</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>